<commit_message>
docs(ai_logs): update Phuc_ai_log.xlsx last updated date (2026-07-21)
</commit_message>
<xml_diff>
--- a/ai_logs/Phuc_ai_log.xlsx
+++ b/ai_logs/Phuc_ai_log.xlsx
@@ -1286,6 +1286,18 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Last Updated:</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>

</xml_diff>